<commit_message>
deprel for 3 sentences
</commit_message>
<xml_diff>
--- a/english.xlsx
+++ b/english.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mamit\Desktop\LT\Computational Syntax\lab3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mamit\Desktop\LT\Computational Syntax\lab3\Universal-Dependencies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7FF1C01-A257-4C41-BF8C-7048A1BC451D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{948BCBFF-5538-4D95-857B-5B5F201CE2DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{11BBC0D1-0CA4-4724-8D54-A31BE93C0D8D}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{11BBC0D1-0CA4-4724-8D54-A31BE93C0D8D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="52">
   <si>
     <t>Who</t>
   </si>
@@ -69,6 +69,132 @@
   </si>
   <si>
     <t>punct</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>small</t>
+  </si>
+  <si>
+    <t>town</t>
+  </si>
+  <si>
+    <t>with</t>
+  </si>
+  <si>
+    <t>two</t>
+  </si>
+  <si>
+    <t>minarets</t>
+  </si>
+  <si>
+    <t>glides</t>
+  </si>
+  <si>
+    <t>by</t>
+  </si>
+  <si>
+    <t>.</t>
+  </si>
+  <si>
+    <t>DET</t>
+  </si>
+  <si>
+    <t>ADJ</t>
+  </si>
+  <si>
+    <t>NOUN</t>
+  </si>
+  <si>
+    <t>ADP</t>
+  </si>
+  <si>
+    <t>NUM</t>
+  </si>
+  <si>
+    <t>VERB</t>
+  </si>
+  <si>
+    <t>ADV</t>
+  </si>
+  <si>
+    <t>det</t>
+  </si>
+  <si>
+    <t>amod</t>
+  </si>
+  <si>
+    <t>case</t>
+  </si>
+  <si>
+    <t>nummod</t>
+  </si>
+  <si>
+    <t>advmod</t>
+  </si>
+  <si>
+    <t>nmod</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>was</t>
+  </si>
+  <si>
+    <t>just</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>boy</t>
+  </si>
+  <si>
+    <t>muddy</t>
+  </si>
+  <si>
+    <t>shoes</t>
+  </si>
+  <si>
+    <t>Shenzhen</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>traffic</t>
+  </si>
+  <si>
+    <t>police</t>
+  </si>
+  <si>
+    <t>have</t>
+  </si>
+  <si>
+    <t>opted</t>
+  </si>
+  <si>
+    <t>for</t>
+  </si>
+  <si>
+    <t>unconventional</t>
+  </si>
+  <si>
+    <t>penalties</t>
+  </si>
+  <si>
+    <t>before</t>
+  </si>
+  <si>
+    <t>PROPN</t>
+  </si>
+  <si>
+    <t>PART</t>
+  </si>
+  <si>
+    <t>cop</t>
   </si>
 </sst>
 </file>
@@ -104,8 +230,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -440,7 +567,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27F2D1FC-F999-4D45-A05E-3DEF813FC2A7}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -454,10 +581,10 @@
         <v>1</v>
       </c>
       <c r="D1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -471,10 +598,10 @@
         <v>4</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>5</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -488,7 +615,7 @@
         <v>1</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="s">
         <v>2</v>
@@ -505,10 +632,463 @@
         <v>8</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <f>A6+1</f>
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <f t="shared" ref="A8:A14" si="0">A7+1</f>
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9">
+        <v>6</v>
+      </c>
+      <c r="E9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10">
+        <v>6</v>
+      </c>
+      <c r="E10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13">
+        <v>7</v>
+      </c>
+      <c r="E13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14">
+        <v>7</v>
+      </c>
+      <c r="E14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>1</v>
+      </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
+      </c>
+      <c r="E16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <f>A16+1</f>
+        <v>2</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" t="s">
+        <v>4</v>
+      </c>
+      <c r="D17">
+        <v>5</v>
+      </c>
+      <c r="E17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <f t="shared" ref="A18:A24" si="1">A17+1</f>
+        <v>3</v>
+      </c>
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18">
+        <v>5</v>
+      </c>
+      <c r="E18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="B19" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19">
+        <v>5</v>
+      </c>
+      <c r="E19" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="B20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" t="s">
+        <v>21</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="B21" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21">
+        <v>8</v>
+      </c>
+      <c r="E21" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="B22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22">
+        <v>8</v>
+      </c>
+      <c r="E22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="B23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23">
+        <v>5</v>
+      </c>
+      <c r="E23" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="B24" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24">
+        <v>5</v>
+      </c>
+      <c r="E24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>1</v>
+      </c>
+      <c r="B26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <f>A26+1</f>
+        <v>2</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <f t="shared" ref="A28:A36" si="2">A27+1</f>
+        <v>3</v>
+      </c>
+      <c r="B28" t="s">
+        <v>41</v>
+      </c>
+      <c r="C28" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="B29" t="s">
+        <v>42</v>
+      </c>
+      <c r="C29" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="B30" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="B31" t="s">
+        <v>44</v>
+      </c>
+      <c r="C31" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="B32" t="s">
+        <v>45</v>
+      </c>
+      <c r="C32" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="B33" t="s">
+        <v>46</v>
+      </c>
+      <c r="C33" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <f t="shared" si="2"/>
+        <v>9</v>
+      </c>
+      <c r="B34" t="s">
+        <v>47</v>
+      </c>
+      <c r="C34" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="B35" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <f t="shared" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="B36" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>